<commit_message>
fix: Kelvin 5/23 entry verified as Garmin
</commit_message>
<xml_diff>
--- a/Reports/Members/Kelvin_Activity_Report.xlsx
+++ b/Reports/Members/Kelvin_Activity_Report.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Garmin</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Committee Approval Required</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>

</xml_diff>